<commit_message>
Data: refresh AA & WM master + Blinkit inventory snapshot
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
+++ b/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Audio Array &amp; WM Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7387449E-FEC1-4802-8131-B7B5E005A4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A678428-CF0E-4B65-8204-F33B36ABAE38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E071ED51-FC72-421D-856E-2A4DF68E7BC3}"/>
   </bookViews>
@@ -3425,6 +3425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98773489-E591-4874-A9C1-F7B78C71D228}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O212"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3491,7 +3492,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -3538,7 +3539,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -3612,7 +3613,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -3649,7 +3650,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -3686,7 +3687,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -3723,7 +3724,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -3760,7 +3761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -3797,7 +3798,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -3834,7 +3835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -3871,7 +3872,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -3908,7 +3909,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -3945,7 +3946,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
@@ -3982,7 +3983,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
@@ -4019,7 +4020,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
@@ -4056,7 +4057,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
@@ -4093,7 +4094,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -4130,7 +4131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
@@ -4165,7 +4166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
@@ -4202,7 +4203,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -4239,7 +4240,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
@@ -4276,7 +4277,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -4313,7 +4314,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>32</v>
       </c>
@@ -4348,7 +4349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>33</v>
       </c>
@@ -4385,7 +4386,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>34</v>
       </c>
@@ -4422,7 +4423,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>35</v>
       </c>
@@ -4459,7 +4460,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>36</v>
       </c>
@@ -4496,7 +4497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>37</v>
       </c>
@@ -4531,7 +4532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>38</v>
       </c>
@@ -4568,7 +4569,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>39</v>
       </c>
@@ -4603,7 +4604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>40</v>
       </c>
@@ -4638,7 +4639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>41</v>
       </c>
@@ -4675,7 +4676,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>42</v>
       </c>
@@ -4712,7 +4713,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>43</v>
       </c>
@@ -4747,7 +4748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>44</v>
       </c>
@@ -4784,7 +4785,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>45</v>
       </c>
@@ -4821,7 +4822,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>46</v>
       </c>
@@ -4858,7 +4859,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>47</v>
       </c>
@@ -4895,7 +4896,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>48</v>
       </c>
@@ -4932,7 +4933,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>49</v>
       </c>
@@ -4969,7 +4970,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>50</v>
       </c>
@@ -5006,7 +5007,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>51</v>
       </c>
@@ -5041,7 +5042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>52</v>
       </c>
@@ -5076,7 +5077,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>53</v>
       </c>
@@ -5113,7 +5114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>54</v>
       </c>
@@ -5150,7 +5151,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>55</v>
       </c>
@@ -5187,7 +5188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>56</v>
       </c>
@@ -5224,7 +5225,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>57</v>
       </c>
@@ -5261,7 +5262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>58</v>
       </c>
@@ -5298,7 +5299,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>59</v>
       </c>
@@ -5335,7 +5336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>60</v>
       </c>
@@ -5372,7 +5373,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>61</v>
       </c>
@@ -5409,7 +5410,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>62</v>
       </c>
@@ -5446,7 +5447,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>63</v>
       </c>
@@ -5483,7 +5484,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>64</v>
       </c>
@@ -5520,7 +5521,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>65</v>
       </c>
@@ -5557,7 +5558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>66</v>
       </c>
@@ -5594,7 +5595,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>67</v>
       </c>
@@ -5631,7 +5632,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>68</v>
       </c>
@@ -5668,7 +5669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>69</v>
       </c>
@@ -5705,7 +5706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>70</v>
       </c>
@@ -5742,7 +5743,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>71</v>
       </c>
@@ -5779,7 +5780,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>72</v>
       </c>
@@ -5816,7 +5817,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>73</v>
       </c>
@@ -5853,7 +5854,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>74</v>
       </c>
@@ -5890,7 +5891,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>75</v>
       </c>
@@ -5927,7 +5928,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>76</v>
       </c>
@@ -5962,7 +5963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>77</v>
       </c>
@@ -5999,7 +6000,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>78</v>
       </c>
@@ -6036,7 +6037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>79</v>
       </c>
@@ -6071,7 +6072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>80</v>
       </c>
@@ -6106,7 +6107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>81</v>
       </c>
@@ -6143,7 +6144,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>82</v>
       </c>
@@ -6180,7 +6181,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>83</v>
       </c>
@@ -6217,7 +6218,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>84</v>
       </c>
@@ -6254,7 +6255,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>85</v>
       </c>
@@ -6291,7 +6292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>86</v>
       </c>
@@ -6328,7 +6329,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>87</v>
       </c>
@@ -6363,7 +6364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>88</v>
       </c>
@@ -6400,7 +6401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>89</v>
       </c>
@@ -6437,7 +6438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>90</v>
       </c>
@@ -6474,7 +6475,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>91</v>
       </c>
@@ -6511,7 +6512,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>92</v>
       </c>
@@ -6548,7 +6549,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>93</v>
       </c>
@@ -6585,7 +6586,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>94</v>
       </c>
@@ -6622,7 +6623,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>95</v>
       </c>
@@ -6659,7 +6660,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>96</v>
       </c>
@@ -6696,7 +6697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>97</v>
       </c>
@@ -6733,7 +6734,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>98</v>
       </c>
@@ -6770,7 +6771,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>99</v>
       </c>
@@ -6807,7 +6808,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>100</v>
       </c>
@@ -6842,7 +6843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>101</v>
       </c>
@@ -6879,7 +6880,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>102</v>
       </c>
@@ -6914,7 +6915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>103</v>
       </c>
@@ -6951,7 +6952,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>104</v>
       </c>
@@ -6986,7 +6987,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>105</v>
       </c>
@@ -7023,7 +7024,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>106</v>
       </c>
@@ -7058,7 +7059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>107</v>
       </c>
@@ -7095,7 +7096,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>108</v>
       </c>
@@ -7132,7 +7133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>109</v>
       </c>
@@ -7169,7 +7170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>110</v>
       </c>
@@ -7206,7 +7207,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>111</v>
       </c>
@@ -7243,7 +7244,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>112</v>
       </c>
@@ -7278,7 +7279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>113</v>
       </c>
@@ -7315,7 +7316,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>114</v>
       </c>
@@ -7352,7 +7353,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>115</v>
       </c>
@@ -7389,7 +7390,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>116</v>
       </c>
@@ -7424,7 +7425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>117</v>
       </c>
@@ -7461,7 +7462,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>118</v>
       </c>
@@ -7496,7 +7497,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>119</v>
       </c>
@@ -7533,7 +7534,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>120</v>
       </c>
@@ -7570,7 +7571,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>121</v>
       </c>
@@ -7605,7 +7606,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>122</v>
       </c>
@@ -7642,7 +7643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>123</v>
       </c>
@@ -7679,7 +7680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>124</v>
       </c>
@@ -7716,7 +7717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>125</v>
       </c>
@@ -7751,7 +7752,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>126</v>
       </c>
@@ -7788,7 +7789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>127</v>
       </c>
@@ -7825,7 +7826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>128</v>
       </c>
@@ -7862,7 +7863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>129</v>
       </c>
@@ -7899,7 +7900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>130</v>
       </c>
@@ -7936,7 +7937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>131</v>
       </c>
@@ -7973,7 +7974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>132</v>
       </c>
@@ -8010,7 +8011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>133</v>
       </c>
@@ -8047,7 +8048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>134</v>
       </c>
@@ -8084,7 +8085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>135</v>
       </c>
@@ -8121,7 +8122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>136</v>
       </c>
@@ -8158,7 +8159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>137</v>
       </c>
@@ -8195,7 +8196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>138</v>
       </c>
@@ -8232,7 +8233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>139</v>
       </c>
@@ -8269,7 +8270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>140</v>
       </c>
@@ -8306,7 +8307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>141</v>
       </c>
@@ -8343,7 +8344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>142</v>
       </c>
@@ -8380,7 +8381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>143</v>
       </c>
@@ -8417,7 +8418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>144</v>
       </c>
@@ -8454,7 +8455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>145</v>
       </c>
@@ -8491,7 +8492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>146</v>
       </c>
@@ -8528,7 +8529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>147</v>
       </c>
@@ -8565,7 +8566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>148</v>
       </c>
@@ -8602,7 +8603,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>149</v>
       </c>
@@ -8639,7 +8640,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>150</v>
       </c>
@@ -8676,7 +8677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>151</v>
       </c>
@@ -8713,7 +8714,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>152</v>
       </c>
@@ -8750,7 +8751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>153</v>
       </c>
@@ -8787,7 +8788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>154</v>
       </c>
@@ -8822,7 +8823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>155</v>
       </c>
@@ -8859,7 +8860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>156</v>
       </c>
@@ -8896,7 +8897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>157</v>
       </c>
@@ -8933,7 +8934,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>158</v>
       </c>
@@ -8970,7 +8971,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>159</v>
       </c>
@@ -9005,7 +9006,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>160</v>
       </c>
@@ -9042,7 +9043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>161</v>
       </c>
@@ -9077,7 +9078,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>162</v>
       </c>
@@ -9114,7 +9115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>163</v>
       </c>
@@ -9151,7 +9152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>164</v>
       </c>
@@ -9186,7 +9187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>165</v>
       </c>
@@ -9223,7 +9224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>166</v>
       </c>
@@ -9260,7 +9261,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>167</v>
       </c>
@@ -9297,7 +9298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>168</v>
       </c>
@@ -9332,7 +9333,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>169</v>
       </c>
@@ -9367,7 +9368,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>170</v>
       </c>
@@ -9404,7 +9405,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>171</v>
       </c>
@@ -9439,7 +9440,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>172</v>
       </c>
@@ -9474,7 +9475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>173</v>
       </c>
@@ -9511,7 +9512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>174</v>
       </c>
@@ -9546,7 +9547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>175</v>
       </c>
@@ -9581,7 +9582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
         <v>176</v>
       </c>
@@ -9616,7 +9617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
         <v>177</v>
       </c>
@@ -9651,7 +9652,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
         <v>178</v>
       </c>
@@ -9686,7 +9687,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
         <v>179</v>
       </c>
@@ -9723,7 +9724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
         <v>180</v>
       </c>
@@ -9758,7 +9759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>181</v>
       </c>
@@ -9793,7 +9794,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
         <v>182</v>
       </c>
@@ -9830,7 +9831,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="1" t="s">
         <v>183</v>
       </c>
@@ -9867,7 +9868,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
         <v>184</v>
       </c>
@@ -9904,7 +9905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>185</v>
       </c>
@@ -9941,7 +9942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
         <v>186</v>
       </c>
@@ -9976,7 +9977,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
         <v>187</v>
       </c>
@@ -10011,7 +10012,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
         <v>188</v>
       </c>
@@ -10048,7 +10049,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
         <v>189</v>
       </c>
@@ -10085,7 +10086,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="1" t="s">
         <v>190</v>
       </c>
@@ -10122,7 +10123,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="1" t="s">
         <v>191</v>
       </c>
@@ -10157,7 +10158,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
         <v>192</v>
       </c>
@@ -10194,7 +10195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" s="1" t="s">
         <v>193</v>
       </c>
@@ -10231,7 +10232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="1" t="s">
         <v>194</v>
       </c>
@@ -10266,7 +10267,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" s="1" t="s">
         <v>195</v>
       </c>
@@ -10301,7 +10302,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>196</v>
       </c>
@@ -10336,7 +10337,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="1" t="s">
         <v>197</v>
       </c>
@@ -10371,7 +10372,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
         <v>198</v>
       </c>
@@ -10406,7 +10407,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="1" t="s">
         <v>199</v>
       </c>
@@ -10443,7 +10444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>200</v>
       </c>
@@ -10478,7 +10479,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="1" t="s">
         <v>201</v>
       </c>
@@ -10513,7 +10514,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" s="1" t="s">
         <v>202</v>
       </c>
@@ -10548,7 +10549,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="1" t="s">
         <v>203</v>
       </c>
@@ -10583,7 +10584,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="1" t="s">
         <v>204</v>
       </c>
@@ -10620,7 +10621,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="1" t="s">
         <v>205</v>
       </c>
@@ -10655,7 +10656,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" s="1" t="s">
         <v>206</v>
       </c>
@@ -10692,7 +10693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="1" t="s">
         <v>207</v>
       </c>
@@ -10727,7 +10728,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="1" t="s">
         <v>208</v>
       </c>
@@ -10762,7 +10763,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="1" t="s">
         <v>209</v>
       </c>
@@ -10799,7 +10800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="1" t="s">
         <v>210</v>
       </c>
@@ -10836,7 +10837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="1" t="s">
         <v>211</v>
       </c>
@@ -10873,7 +10874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="1" t="s">
         <v>212</v>
       </c>
@@ -10910,7 +10911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="1" t="s">
         <v>213</v>
       </c>
@@ -10945,7 +10946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" s="1" t="s">
         <v>214</v>
       </c>
@@ -10980,7 +10981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" s="1" t="s">
         <v>215</v>
       </c>
@@ -11015,7 +11016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" s="1" t="s">
         <v>216</v>
       </c>
@@ -11050,7 +11051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" s="1" t="s">
         <v>217</v>
       </c>
@@ -11085,7 +11086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" s="1" t="s">
         <v>218</v>
       </c>
@@ -11120,7 +11121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" s="1" t="s">
         <v>219</v>
       </c>
@@ -11160,7 +11161,13 @@
       <c r="B212" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O211" xr:uid="{98773489-E591-4874-A9C1-F7B78C71D228}"/>
+  <autoFilter ref="A1:O211" xr:uid="{98773489-E591-4874-A9C1-F7B78C71D228}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="AM-S1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="A3">
     <cfRule type="duplicateValues" dxfId="50" priority="102"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Data: align AA/WM/CB/Nexlev/Viomi replenishment masters with sku_master
Refreshed master sheets so every SKU resolves to sku_master and every
Model matches (case-insensitive). Audit against the canonical
G:/...master/sku_master.xlsx now reports 0 mismatches across all 5
replenishment scopes (AA 210, WM 44, CB 236, Nexlev 112, Viomi 112).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
+++ b/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Audio Array &amp; WM Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A678428-CF0E-4B65-8204-F33B36ABAE38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48138569-E608-42B2-911B-A4F5C94C9E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E071ED51-FC72-421D-856E-2A4DF68E7BC3}"/>
   </bookViews>
@@ -3425,7 +3425,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98773489-E591-4874-A9C1-F7B78C71D228}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:O212"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3492,7 +3491,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -3539,7 +3538,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -3613,7 +3612,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -3650,7 +3649,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -3687,7 +3686,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -3724,7 +3723,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -3761,7 +3760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -3798,7 +3797,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -3835,7 +3834,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -3872,7 +3871,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -3909,7 +3908,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -3946,7 +3945,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
@@ -3983,7 +3982,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
@@ -4020,7 +4019,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
@@ -4057,7 +4056,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
@@ -4094,7 +4093,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -4131,7 +4130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
@@ -4166,7 +4165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
@@ -4203,7 +4202,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -4240,7 +4239,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
@@ -4277,7 +4276,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -4314,7 +4313,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>32</v>
       </c>
@@ -4349,7 +4348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>33</v>
       </c>
@@ -4386,7 +4385,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>34</v>
       </c>
@@ -4423,7 +4422,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>35</v>
       </c>
@@ -4460,7 +4459,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>36</v>
       </c>
@@ -4497,7 +4496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>37</v>
       </c>
@@ -4532,7 +4531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>38</v>
       </c>
@@ -4569,7 +4568,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>39</v>
       </c>
@@ -4604,7 +4603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>40</v>
       </c>
@@ -4639,7 +4638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>41</v>
       </c>
@@ -4676,7 +4675,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>42</v>
       </c>
@@ -4713,7 +4712,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>43</v>
       </c>
@@ -4748,7 +4747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>44</v>
       </c>
@@ -4785,7 +4784,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>45</v>
       </c>
@@ -4822,7 +4821,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>46</v>
       </c>
@@ -4859,7 +4858,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>47</v>
       </c>
@@ -4896,7 +4895,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>48</v>
       </c>
@@ -4933,7 +4932,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>49</v>
       </c>
@@ -4970,7 +4969,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="42" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>50</v>
       </c>
@@ -5007,7 +5006,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>51</v>
       </c>
@@ -5042,7 +5041,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>52</v>
       </c>
@@ -5077,7 +5076,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>53</v>
       </c>
@@ -5114,7 +5113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>54</v>
       </c>
@@ -5151,7 +5150,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>55</v>
       </c>
@@ -5188,7 +5187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>56</v>
       </c>
@@ -5225,7 +5224,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="49" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>57</v>
       </c>
@@ -5262,7 +5261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>58</v>
       </c>
@@ -5299,7 +5298,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>59</v>
       </c>
@@ -5336,7 +5335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>60</v>
       </c>
@@ -5373,7 +5372,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="53" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>61</v>
       </c>
@@ -5410,7 +5409,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>62</v>
       </c>
@@ -5447,7 +5446,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>63</v>
       </c>
@@ -5484,7 +5483,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>64</v>
       </c>
@@ -5521,7 +5520,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>65</v>
       </c>
@@ -5558,7 +5557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>66</v>
       </c>
@@ -5595,7 +5594,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="59" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>67</v>
       </c>
@@ -5632,7 +5631,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>68</v>
       </c>
@@ -5669,7 +5668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>69</v>
       </c>
@@ -5706,7 +5705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>70</v>
       </c>
@@ -5743,7 +5742,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>71</v>
       </c>
@@ -5780,7 +5779,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>72</v>
       </c>
@@ -5817,7 +5816,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>73</v>
       </c>
@@ -5854,7 +5853,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="66" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>74</v>
       </c>
@@ -5891,7 +5890,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="67" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>75</v>
       </c>
@@ -5928,7 +5927,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="68" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>76</v>
       </c>
@@ -5963,7 +5962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>77</v>
       </c>
@@ -6000,7 +5999,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>78</v>
       </c>
@@ -6037,7 +6036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>79</v>
       </c>
@@ -6072,7 +6071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>80</v>
       </c>
@@ -6107,7 +6106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>81</v>
       </c>
@@ -6144,7 +6143,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="74" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>82</v>
       </c>
@@ -6181,7 +6180,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="75" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>83</v>
       </c>
@@ -6218,7 +6217,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="76" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>84</v>
       </c>
@@ -6255,7 +6254,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="77" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>85</v>
       </c>
@@ -6292,7 +6291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>86</v>
       </c>
@@ -6329,7 +6328,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>87</v>
       </c>
@@ -6364,7 +6363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>88</v>
       </c>
@@ -6401,7 +6400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>89</v>
       </c>
@@ -6438,7 +6437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>90</v>
       </c>
@@ -6475,7 +6474,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="83" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>91</v>
       </c>
@@ -6512,7 +6511,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>92</v>
       </c>
@@ -6549,7 +6548,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>93</v>
       </c>
@@ -6586,7 +6585,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>94</v>
       </c>
@@ -6623,7 +6622,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>95</v>
       </c>
@@ -6660,7 +6659,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="88" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>96</v>
       </c>
@@ -6697,7 +6696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>97</v>
       </c>
@@ -6734,7 +6733,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>98</v>
       </c>
@@ -6771,7 +6770,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>99</v>
       </c>
@@ -6808,7 +6807,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>100</v>
       </c>
@@ -6843,7 +6842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>101</v>
       </c>
@@ -6880,7 +6879,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="94" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>102</v>
       </c>
@@ -6915,7 +6914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>103</v>
       </c>
@@ -6952,7 +6951,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>104</v>
       </c>
@@ -6987,7 +6986,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="97" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>105</v>
       </c>
@@ -7024,7 +7023,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="98" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>106</v>
       </c>
@@ -7059,7 +7058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>107</v>
       </c>
@@ -7096,7 +7095,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="100" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>108</v>
       </c>
@@ -7133,7 +7132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>109</v>
       </c>
@@ -7170,7 +7169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>110</v>
       </c>
@@ -7207,7 +7206,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="103" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>111</v>
       </c>
@@ -7244,7 +7243,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="104" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>112</v>
       </c>
@@ -7279,7 +7278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>113</v>
       </c>
@@ -7316,7 +7315,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>114</v>
       </c>
@@ -7353,7 +7352,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="107" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>115</v>
       </c>
@@ -7390,7 +7389,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="108" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>116</v>
       </c>
@@ -7425,7 +7424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>117</v>
       </c>
@@ -7462,7 +7461,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="110" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>118</v>
       </c>
@@ -7497,7 +7496,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="111" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>119</v>
       </c>
@@ -7534,7 +7533,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="112" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>120</v>
       </c>
@@ -7571,7 +7570,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="113" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>121</v>
       </c>
@@ -7606,7 +7605,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="114" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>122</v>
       </c>
@@ -7643,7 +7642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>123</v>
       </c>
@@ -7680,7 +7679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>124</v>
       </c>
@@ -7717,7 +7716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>125</v>
       </c>
@@ -7752,7 +7751,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="118" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>126</v>
       </c>
@@ -7789,7 +7788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>127</v>
       </c>
@@ -7826,7 +7825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>128</v>
       </c>
@@ -7863,7 +7862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>129</v>
       </c>
@@ -7900,7 +7899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>130</v>
       </c>
@@ -7937,7 +7936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>131</v>
       </c>
@@ -7974,7 +7973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>132</v>
       </c>
@@ -8011,7 +8010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>133</v>
       </c>
@@ -8048,7 +8047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>134</v>
       </c>
@@ -8085,7 +8084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>135</v>
       </c>
@@ -8122,7 +8121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>136</v>
       </c>
@@ -8159,7 +8158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>137</v>
       </c>
@@ -8196,7 +8195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>138</v>
       </c>
@@ -8233,7 +8232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>139</v>
       </c>
@@ -8270,7 +8269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>140</v>
       </c>
@@ -8307,7 +8306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>141</v>
       </c>
@@ -8344,7 +8343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>142</v>
       </c>
@@ -8381,7 +8380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>143</v>
       </c>
@@ -8418,7 +8417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>144</v>
       </c>
@@ -8455,7 +8454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>145</v>
       </c>
@@ -8492,7 +8491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>146</v>
       </c>
@@ -8529,7 +8528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>147</v>
       </c>
@@ -8566,7 +8565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>148</v>
       </c>
@@ -8603,7 +8602,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="141" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>149</v>
       </c>
@@ -8640,7 +8639,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="142" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>150</v>
       </c>
@@ -8677,7 +8676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>151</v>
       </c>
@@ -8714,7 +8713,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="144" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>152</v>
       </c>
@@ -8751,7 +8750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>153</v>
       </c>
@@ -8788,7 +8787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>154</v>
       </c>
@@ -8823,7 +8822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>155</v>
       </c>
@@ -8860,7 +8859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>156</v>
       </c>
@@ -8897,7 +8896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>157</v>
       </c>
@@ -8934,7 +8933,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="150" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>158</v>
       </c>
@@ -8971,7 +8970,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="151" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>159</v>
       </c>
@@ -9006,7 +9005,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>160</v>
       </c>
@@ -9043,7 +9042,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="153" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>161</v>
       </c>
@@ -9078,7 +9077,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="154" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>162</v>
       </c>
@@ -9115,7 +9114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>163</v>
       </c>
@@ -9152,7 +9151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>164</v>
       </c>
@@ -9187,7 +9186,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>165</v>
       </c>
@@ -9224,7 +9223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>166</v>
       </c>
@@ -9261,7 +9260,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="159" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>167</v>
       </c>
@@ -9298,7 +9297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>168</v>
       </c>
@@ -9333,7 +9332,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="161" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>169</v>
       </c>
@@ -9368,7 +9367,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="162" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>170</v>
       </c>
@@ -9405,7 +9404,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="163" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>171</v>
       </c>
@@ -9440,7 +9439,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>172</v>
       </c>
@@ -9475,7 +9474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>173</v>
       </c>
@@ -9512,7 +9511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>174</v>
       </c>
@@ -9547,7 +9546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>175</v>
       </c>
@@ -9582,7 +9581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
         <v>176</v>
       </c>
@@ -9617,7 +9616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
         <v>177</v>
       </c>
@@ -9652,7 +9651,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="170" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
         <v>178</v>
       </c>
@@ -9687,7 +9686,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="171" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
         <v>179</v>
       </c>
@@ -9724,7 +9723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
         <v>180</v>
       </c>
@@ -9759,7 +9758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>181</v>
       </c>
@@ -9794,7 +9793,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="174" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
         <v>182</v>
       </c>
@@ -9831,7 +9830,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="175" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A175" s="1" t="s">
         <v>183</v>
       </c>
@@ -9868,7 +9867,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="176" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
         <v>184</v>
       </c>
@@ -9905,7 +9904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>185</v>
       </c>
@@ -9942,7 +9941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
         <v>186</v>
       </c>
@@ -9977,7 +9976,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="179" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
         <v>187</v>
       </c>
@@ -10012,7 +10011,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="180" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
         <v>188</v>
       </c>
@@ -10049,7 +10048,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="181" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
         <v>189</v>
       </c>
@@ -10086,7 +10085,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="182" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A182" s="1" t="s">
         <v>190</v>
       </c>
@@ -10123,7 +10122,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="183" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A183" s="1" t="s">
         <v>191</v>
       </c>
@@ -10158,7 +10157,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="184" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
         <v>192</v>
       </c>
@@ -10195,7 +10194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A185" s="1" t="s">
         <v>193</v>
       </c>
@@ -10232,7 +10231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A186" s="1" t="s">
         <v>194</v>
       </c>
@@ -10267,7 +10266,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="187" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A187" s="1" t="s">
         <v>195</v>
       </c>
@@ -10302,7 +10301,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="188" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>196</v>
       </c>
@@ -10337,7 +10336,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="189" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A189" s="1" t="s">
         <v>197</v>
       </c>
@@ -10372,7 +10371,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="190" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
         <v>198</v>
       </c>
@@ -10407,7 +10406,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="191" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A191" s="1" t="s">
         <v>199</v>
       </c>
@@ -10444,7 +10443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>200</v>
       </c>
@@ -10479,7 +10478,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="193" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A193" s="1" t="s">
         <v>201</v>
       </c>
@@ -10514,7 +10513,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="194" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A194" s="1" t="s">
         <v>202</v>
       </c>
@@ -10549,7 +10548,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="195" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A195" s="1" t="s">
         <v>203</v>
       </c>
@@ -10584,7 +10583,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="196" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A196" s="1" t="s">
         <v>204</v>
       </c>
@@ -10621,7 +10620,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="197" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A197" s="1" t="s">
         <v>205</v>
       </c>
@@ -10656,7 +10655,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="198" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A198" s="1" t="s">
         <v>206</v>
       </c>
@@ -10693,7 +10692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A199" s="1" t="s">
         <v>207</v>
       </c>
@@ -10728,7 +10727,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="200" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A200" s="1" t="s">
         <v>208</v>
       </c>
@@ -10763,7 +10762,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="201" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A201" s="1" t="s">
         <v>209</v>
       </c>
@@ -10800,7 +10799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A202" s="1" t="s">
         <v>210</v>
       </c>
@@ -10837,7 +10836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A203" s="1" t="s">
         <v>211</v>
       </c>
@@ -10874,7 +10873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A204" s="1" t="s">
         <v>212</v>
       </c>
@@ -10911,7 +10910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A205" s="1" t="s">
         <v>213</v>
       </c>
@@ -10946,7 +10945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A206" s="1" t="s">
         <v>214</v>
       </c>
@@ -10981,7 +10980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A207" s="1" t="s">
         <v>215</v>
       </c>
@@ -11016,7 +11015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A208" s="1" t="s">
         <v>216</v>
       </c>
@@ -11051,7 +11050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A209" s="1" t="s">
         <v>217</v>
       </c>
@@ -11086,7 +11085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A210" s="1" t="s">
         <v>218</v>
       </c>
@@ -11121,7 +11120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A211" s="1" t="s">
         <v>219</v>
       </c>
@@ -11161,13 +11160,6 @@
       <c r="B212" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O211" xr:uid="{98773489-E591-4874-A9C1-F7B78C71D228}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="AM-S1"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <conditionalFormatting sqref="A3">
     <cfRule type="duplicateValues" dxfId="50" priority="102"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Viomi SP-API inbound + AA/WM V3 + Nexlev/Viomi master refresh
- inbound_shipments_viomi.csv: first SP-API pull via AM Replenishment
  Inbound app (84 rows / 26 active shipments / 1,364 incoming units
  to ISK3 + DEL4 + HYD3 + others).
- AA & WM Replenishment.xlsx: V3 — adds 39 AA SKUs + 1 WM SKU
  (FBA79175 WM-SMD09-WH); 5 AA model renames; 4 master-carton fills.
- replenishment_master_nexlev.xlsx + viomi.xlsx: operator weekly refresh.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
+++ b/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Audio Array &amp; WM Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41946D65-06A5-410B-909E-CDCAEA29C259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A72F9A0-4253-4F0D-B581-67E62C2F8BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E071ED51-FC72-421D-856E-2A4DF68E7BC3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1672" uniqueCount="842">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1681" uniqueCount="845">
   <si>
     <t>SKU</t>
   </si>
@@ -2565,6 +2565,15 @@
   </si>
   <si>
     <t>B0H1MTP2ZP</t>
+  </si>
+  <si>
+    <t>FBA79175</t>
+  </si>
+  <si>
+    <t>B0CPT2YJX2</t>
+  </si>
+  <si>
+    <t>WM-SMD09-WH</t>
   </si>
 </sst>
 </file>
@@ -2627,7 +2636,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -2663,12 +2672,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2703,6 +2723,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -11539,19 +11562,19 @@
     <cfRule type="duplicateValues" dxfId="39" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A107">
-    <cfRule type="duplicateValues" dxfId="38" priority="115"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A108:A110">
-    <cfRule type="duplicateValues" dxfId="36" priority="117"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="117"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A112:A134">
     <cfRule type="duplicateValues" dxfId="34" priority="119"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A138">
-    <cfRule type="duplicateValues" dxfId="33" priority="120"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="121"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="121"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="120"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A147:A155">
     <cfRule type="duplicateValues" dxfId="31" priority="122"/>
@@ -11601,8 +11624,8 @@
     <cfRule type="duplicateValues" dxfId="15" priority="86"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B140">
-    <cfRule type="duplicateValues" dxfId="14" priority="67"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B141">
     <cfRule type="duplicateValues" dxfId="12" priority="69"/>
@@ -11634,7 +11657,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0CFBFCC-8DAC-4EC0-9F68-2F31D96435DD}">
-  <dimension ref="A1:R43"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
@@ -13394,6 +13417,38 @@
       </c>
       <c r="R43" t="s">
         <v>762</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>842</v>
+      </c>
+      <c r="B44" t="s">
+        <v>843</v>
+      </c>
+      <c r="C44" t="s">
+        <v>844</v>
+      </c>
+      <c r="D44" t="s">
+        <v>739</v>
+      </c>
+      <c r="E44" t="s">
+        <v>742</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>756</v>
+      </c>
+      <c r="O44" s="13">
+        <v>1</v>
+      </c>
+      <c r="P44" t="s">
+        <v>758</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>763</v>
+      </c>
+      <c r="R44" t="s">
+        <v>763</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AA repl-master expansion (V3) + sku_master backfill (FBA80181)
- AA sheet: 222 -> 262 rows (39 new SKUs from V3 — AM-W series whiteboards,
  AK-S1/S2, AB-06..09, plus FBA80006 / FBA80109+ family).
- sku_master: +1 SKU (FBA80181).

Known gap (not blocking — to triage with data team): 13 SKUs in AA sheet
are still missing from sku_master:
  FBA76709-14, FBA76731 (AM-W38..44),
  FBA79006-7 (AK-S1, AK-S2),
  FBA79326-29 (AB-06..09).
Audit will flag these until master is updated. Many have valid ASINs
(B0BLJYX15C / B0BLK1Z7PJ / B0BLK9QL7X / B0CYLXLBRL / B0CYLVB618 /
B0CYLXL5GY / B0CYLXC8BQ); others are "ASIN Not created" — handle when
listings go live.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
+++ b/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Audio Array &amp; WM Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A72F9A0-4253-4F0D-B581-67E62C2F8BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2476F9D6-173C-4C5E-9AFB-64CF57A0789A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E071ED51-FC72-421D-856E-2A4DF68E7BC3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E071ED51-FC72-421D-856E-2A4DF68E7BC3}"/>
   </bookViews>
   <sheets>
     <sheet name="AA" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1681" uniqueCount="845">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="935">
   <si>
     <t>SKU</t>
   </si>
@@ -2574,6 +2574,276 @@
   </si>
   <si>
     <t>WM-SMD09-WH</t>
+  </si>
+  <si>
+    <t>FBA80006</t>
+  </si>
+  <si>
+    <t>FBA76731</t>
+  </si>
+  <si>
+    <t>FBA76713</t>
+  </si>
+  <si>
+    <t>FBA76709</t>
+  </si>
+  <si>
+    <t>FBA76710</t>
+  </si>
+  <si>
+    <t>FBA76711</t>
+  </si>
+  <si>
+    <t>FBA76712</t>
+  </si>
+  <si>
+    <t>FBA76714</t>
+  </si>
+  <si>
+    <t>FBA79006</t>
+  </si>
+  <si>
+    <t>FBA79007</t>
+  </si>
+  <si>
+    <t>FBA79326</t>
+  </si>
+  <si>
+    <t>FBA79327</t>
+  </si>
+  <si>
+    <t>FBA79328</t>
+  </si>
+  <si>
+    <t>FBA79329</t>
+  </si>
+  <si>
+    <t>FBA80109</t>
+  </si>
+  <si>
+    <t>FBA80110</t>
+  </si>
+  <si>
+    <t>FBA80119</t>
+  </si>
+  <si>
+    <t>FBA80120</t>
+  </si>
+  <si>
+    <t>FBA80121</t>
+  </si>
+  <si>
+    <t>FBA80122</t>
+  </si>
+  <si>
+    <t>FBA80123</t>
+  </si>
+  <si>
+    <t>FBA80124</t>
+  </si>
+  <si>
+    <t>FBA80125</t>
+  </si>
+  <si>
+    <t>FBA80126</t>
+  </si>
+  <si>
+    <t>FBA80129</t>
+  </si>
+  <si>
+    <t>FBA80130</t>
+  </si>
+  <si>
+    <t>FBA80131</t>
+  </si>
+  <si>
+    <t>FBA80132</t>
+  </si>
+  <si>
+    <t>FBA80133</t>
+  </si>
+  <si>
+    <t>FBA80134</t>
+  </si>
+  <si>
+    <t>FBA80135</t>
+  </si>
+  <si>
+    <t>FBA80136</t>
+  </si>
+  <si>
+    <t>FBA80137</t>
+  </si>
+  <si>
+    <t>FBA80138</t>
+  </si>
+  <si>
+    <t>FBA80142</t>
+  </si>
+  <si>
+    <t>FBA80114</t>
+  </si>
+  <si>
+    <t>FBA80115</t>
+  </si>
+  <si>
+    <t>FBA80116</t>
+  </si>
+  <si>
+    <t>FBA80117</t>
+  </si>
+  <si>
+    <t>ASIN Not created</t>
+  </si>
+  <si>
+    <t>B0BLK9QL7X</t>
+  </si>
+  <si>
+    <t>B0BLK1Z7PJ</t>
+  </si>
+  <si>
+    <t>B0BLJYX15C</t>
+  </si>
+  <si>
+    <t>B0CYLXLBRL</t>
+  </si>
+  <si>
+    <t>B0CYLVB618</t>
+  </si>
+  <si>
+    <t>B0CYLXL5GY</t>
+  </si>
+  <si>
+    <t>B0CYLXC8BQ</t>
+  </si>
+  <si>
+    <t>B0H2ZCQFTZ</t>
+  </si>
+  <si>
+    <t>B0H2Z6R6V8</t>
+  </si>
+  <si>
+    <t>B0H3LHF2WW</t>
+  </si>
+  <si>
+    <t>A2-XLR</t>
+  </si>
+  <si>
+    <t>AM-W48</t>
+  </si>
+  <si>
+    <t>AM-W44</t>
+  </si>
+  <si>
+    <t>AM-W42</t>
+  </si>
+  <si>
+    <t>AM-W38</t>
+  </si>
+  <si>
+    <t>AM-W39</t>
+  </si>
+  <si>
+    <t>AM-W40</t>
+  </si>
+  <si>
+    <t>AM-W41</t>
+  </si>
+  <si>
+    <t>AM-W43</t>
+  </si>
+  <si>
+    <t>AK-S1</t>
+  </si>
+  <si>
+    <t>AK-S2</t>
+  </si>
+  <si>
+    <t>AB-06</t>
+  </si>
+  <si>
+    <t>AB-07</t>
+  </si>
+  <si>
+    <t>AB-08</t>
+  </si>
+  <si>
+    <t>AB-09</t>
+  </si>
+  <si>
+    <t>M5</t>
+  </si>
+  <si>
+    <t>X5</t>
+  </si>
+  <si>
+    <t>AM-C53</t>
+  </si>
+  <si>
+    <t>AM-C54</t>
+  </si>
+  <si>
+    <t>AM-C55</t>
+  </si>
+  <si>
+    <t>AM-C56</t>
+  </si>
+  <si>
+    <t>AM-W25</t>
+  </si>
+  <si>
+    <t>AA-26 Pro</t>
+  </si>
+  <si>
+    <t>AA-27</t>
+  </si>
+  <si>
+    <t>AA-28</t>
+  </si>
+  <si>
+    <t>HP4</t>
+  </si>
+  <si>
+    <t>HPA1400</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>PRE103</t>
+  </si>
+  <si>
+    <t>DI20</t>
+  </si>
+  <si>
+    <t>AC1</t>
+  </si>
+  <si>
+    <t>IS-2</t>
+  </si>
+  <si>
+    <t>IS-3</t>
+  </si>
+  <si>
+    <t>P7</t>
+  </si>
+  <si>
+    <t>MS155</t>
+  </si>
+  <si>
+    <t>AM-C5 White</t>
+  </si>
+  <si>
+    <t>AH-53</t>
+  </si>
+  <si>
+    <t>AH-50-DH</t>
+  </si>
+  <si>
+    <t>AH-40 Pro</t>
+  </si>
+  <si>
+    <t>AH-53 Pro</t>
   </si>
 </sst>
 </file>
@@ -2688,7 +2958,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2724,9 +2994,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3553,7 +3824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98773489-E591-4874-A9C1-F7B78C71D228}">
-  <dimension ref="A1:O223"/>
+  <dimension ref="A1:O263"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -11302,6 +11573,9 @@
       <c r="I212" s="2">
         <v>0</v>
       </c>
+      <c r="O212" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="213" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
@@ -11322,6 +11596,9 @@
       <c r="I213" s="2">
         <v>0</v>
       </c>
+      <c r="O213" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="214" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
@@ -11342,6 +11619,9 @@
       <c r="I214" s="2">
         <v>0</v>
       </c>
+      <c r="O214" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="215" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
@@ -11362,6 +11642,9 @@
       <c r="I215" s="2">
         <v>0</v>
       </c>
+      <c r="O215" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="216" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
@@ -11382,6 +11665,9 @@
       <c r="I216" s="2">
         <v>0</v>
       </c>
+      <c r="O216" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="217" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
@@ -11402,6 +11688,9 @@
       <c r="I217" s="2">
         <v>0</v>
       </c>
+      <c r="O217" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="218" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
@@ -11422,6 +11711,9 @@
       <c r="I218" s="2">
         <v>0</v>
       </c>
+      <c r="O218" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="219" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
@@ -11442,6 +11734,9 @@
       <c r="I219" s="2">
         <v>0</v>
       </c>
+      <c r="O219" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="220" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
@@ -11462,6 +11757,9 @@
       <c r="I220" s="2">
         <v>0</v>
       </c>
+      <c r="O220" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="221" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
@@ -11482,6 +11780,9 @@
       <c r="I221" s="2">
         <v>0</v>
       </c>
+      <c r="O221" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="222" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
@@ -11502,6 +11803,9 @@
       <c r="I222" s="2">
         <v>0</v>
       </c>
+      <c r="O222" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="223" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
@@ -11520,6 +11824,809 @@
         <v>610</v>
       </c>
       <c r="I223" s="2">
+        <v>0</v>
+      </c>
+      <c r="O223" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>845</v>
+      </c>
+      <c r="B224" t="s">
+        <v>884</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D224" t="s">
+        <v>895</v>
+      </c>
+      <c r="F224" t="s">
+        <v>610</v>
+      </c>
+      <c r="O224" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>154</v>
+      </c>
+      <c r="B225" t="s">
+        <v>605</v>
+      </c>
+      <c r="C225" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D225" t="s">
+        <v>896</v>
+      </c>
+      <c r="F225" t="s">
+        <v>610</v>
+      </c>
+      <c r="O225" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>846</v>
+      </c>
+      <c r="B226" t="s">
+        <v>885</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D226" t="s">
+        <v>897</v>
+      </c>
+      <c r="F226" t="s">
+        <v>610</v>
+      </c>
+      <c r="O226" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>847</v>
+      </c>
+      <c r="B227" t="s">
+        <v>886</v>
+      </c>
+      <c r="C227" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D227" t="s">
+        <v>898</v>
+      </c>
+      <c r="F227" t="s">
+        <v>610</v>
+      </c>
+      <c r="O227" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>848</v>
+      </c>
+      <c r="B228" t="s">
+        <v>887</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D228" t="s">
+        <v>899</v>
+      </c>
+      <c r="F228" t="s">
+        <v>610</v>
+      </c>
+      <c r="O228" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>849</v>
+      </c>
+      <c r="B229" t="s">
+        <v>884</v>
+      </c>
+      <c r="C229" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D229" t="s">
+        <v>900</v>
+      </c>
+      <c r="F229" t="s">
+        <v>610</v>
+      </c>
+      <c r="O229" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>850</v>
+      </c>
+      <c r="B230" t="s">
+        <v>884</v>
+      </c>
+      <c r="C230" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D230" t="s">
+        <v>901</v>
+      </c>
+      <c r="F230" t="s">
+        <v>610</v>
+      </c>
+      <c r="O230" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>851</v>
+      </c>
+      <c r="B231" t="s">
+        <v>884</v>
+      </c>
+      <c r="C231" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D231" t="s">
+        <v>902</v>
+      </c>
+      <c r="F231" t="s">
+        <v>610</v>
+      </c>
+      <c r="O231" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>852</v>
+      </c>
+      <c r="B232" t="s">
+        <v>884</v>
+      </c>
+      <c r="C232" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D232" t="s">
+        <v>903</v>
+      </c>
+      <c r="F232" t="s">
+        <v>610</v>
+      </c>
+      <c r="O232" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>853</v>
+      </c>
+      <c r="B233" t="s">
+        <v>884</v>
+      </c>
+      <c r="C233" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D233" t="s">
+        <v>904</v>
+      </c>
+      <c r="F233" t="s">
+        <v>610</v>
+      </c>
+      <c r="O233" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>854</v>
+      </c>
+      <c r="B234" t="s">
+        <v>884</v>
+      </c>
+      <c r="C234" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D234" t="s">
+        <v>905</v>
+      </c>
+      <c r="F234" t="s">
+        <v>610</v>
+      </c>
+      <c r="O234" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>855</v>
+      </c>
+      <c r="B235" t="s">
+        <v>888</v>
+      </c>
+      <c r="C235" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D235" t="s">
+        <v>906</v>
+      </c>
+      <c r="F235" t="s">
+        <v>610</v>
+      </c>
+      <c r="O235" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>856</v>
+      </c>
+      <c r="B236" t="s">
+        <v>889</v>
+      </c>
+      <c r="C236" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D236" t="s">
+        <v>907</v>
+      </c>
+      <c r="F236" t="s">
+        <v>610</v>
+      </c>
+      <c r="O236" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>857</v>
+      </c>
+      <c r="B237" t="s">
+        <v>890</v>
+      </c>
+      <c r="C237" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D237" t="s">
+        <v>908</v>
+      </c>
+      <c r="F237" t="s">
+        <v>610</v>
+      </c>
+      <c r="O237" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>858</v>
+      </c>
+      <c r="B238" t="s">
+        <v>891</v>
+      </c>
+      <c r="C238" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D238" t="s">
+        <v>909</v>
+      </c>
+      <c r="F238" t="s">
+        <v>610</v>
+      </c>
+      <c r="O238" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>859</v>
+      </c>
+      <c r="B239" t="s">
+        <v>892</v>
+      </c>
+      <c r="C239" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D239" t="s">
+        <v>910</v>
+      </c>
+      <c r="F239" t="s">
+        <v>610</v>
+      </c>
+      <c r="O239" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>860</v>
+      </c>
+      <c r="B240" t="s">
+        <v>893</v>
+      </c>
+      <c r="C240" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D240" t="s">
+        <v>911</v>
+      </c>
+      <c r="F240" t="s">
+        <v>610</v>
+      </c>
+      <c r="O240" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A241" t="s">
+        <v>861</v>
+      </c>
+      <c r="B241" t="s">
+        <v>884</v>
+      </c>
+      <c r="C241" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D241" t="s">
+        <v>912</v>
+      </c>
+      <c r="F241" t="s">
+        <v>610</v>
+      </c>
+      <c r="O241" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A242" t="s">
+        <v>862</v>
+      </c>
+      <c r="B242" t="s">
+        <v>884</v>
+      </c>
+      <c r="C242" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D242" t="s">
+        <v>913</v>
+      </c>
+      <c r="F242" t="s">
+        <v>610</v>
+      </c>
+      <c r="O242" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A243" t="s">
+        <v>863</v>
+      </c>
+      <c r="B243" t="s">
+        <v>884</v>
+      </c>
+      <c r="C243" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D243" t="s">
+        <v>914</v>
+      </c>
+      <c r="F243" t="s">
+        <v>610</v>
+      </c>
+      <c r="O243" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A244" t="s">
+        <v>864</v>
+      </c>
+      <c r="B244" t="s">
+        <v>884</v>
+      </c>
+      <c r="C244" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D244" t="s">
+        <v>915</v>
+      </c>
+      <c r="F244" t="s">
+        <v>610</v>
+      </c>
+      <c r="O244" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A245" t="s">
+        <v>865</v>
+      </c>
+      <c r="B245" t="s">
+        <v>884</v>
+      </c>
+      <c r="C245" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D245" t="s">
+        <v>916</v>
+      </c>
+      <c r="F245" t="s">
+        <v>610</v>
+      </c>
+      <c r="O245" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A246" t="s">
+        <v>866</v>
+      </c>
+      <c r="B246" t="s">
+        <v>884</v>
+      </c>
+      <c r="C246" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D246" t="s">
+        <v>917</v>
+      </c>
+      <c r="F246" t="s">
+        <v>610</v>
+      </c>
+      <c r="O246" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A247" t="s">
+        <v>867</v>
+      </c>
+      <c r="B247" t="s">
+        <v>884</v>
+      </c>
+      <c r="C247" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D247" t="s">
+        <v>918</v>
+      </c>
+      <c r="F247" t="s">
+        <v>610</v>
+      </c>
+      <c r="O247" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A248" t="s">
+        <v>868</v>
+      </c>
+      <c r="B248" t="s">
+        <v>884</v>
+      </c>
+      <c r="C248" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D248" t="s">
+        <v>919</v>
+      </c>
+      <c r="F248" t="s">
+        <v>610</v>
+      </c>
+      <c r="O248" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A249" t="s">
+        <v>869</v>
+      </c>
+      <c r="B249" t="s">
+        <v>884</v>
+      </c>
+      <c r="C249" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D249" t="s">
+        <v>920</v>
+      </c>
+      <c r="F249" t="s">
+        <v>610</v>
+      </c>
+      <c r="O249" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A250" t="s">
+        <v>870</v>
+      </c>
+      <c r="B250" t="s">
+        <v>884</v>
+      </c>
+      <c r="C250" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D250" t="s">
+        <v>921</v>
+      </c>
+      <c r="F250" t="s">
+        <v>610</v>
+      </c>
+      <c r="O250" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A251" t="s">
+        <v>871</v>
+      </c>
+      <c r="B251" t="s">
+        <v>884</v>
+      </c>
+      <c r="C251" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D251" t="s">
+        <v>922</v>
+      </c>
+      <c r="F251" t="s">
+        <v>610</v>
+      </c>
+      <c r="O251" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A252" t="s">
+        <v>872</v>
+      </c>
+      <c r="B252" t="s">
+        <v>884</v>
+      </c>
+      <c r="C252" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D252" t="s">
+        <v>923</v>
+      </c>
+      <c r="F252" t="s">
+        <v>610</v>
+      </c>
+      <c r="O252" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A253" t="s">
+        <v>873</v>
+      </c>
+      <c r="B253" t="s">
+        <v>884</v>
+      </c>
+      <c r="C253" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D253" t="s">
+        <v>924</v>
+      </c>
+      <c r="F253" t="s">
+        <v>610</v>
+      </c>
+      <c r="O253" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A254" t="s">
+        <v>874</v>
+      </c>
+      <c r="B254" t="s">
+        <v>884</v>
+      </c>
+      <c r="C254" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D254" t="s">
+        <v>925</v>
+      </c>
+      <c r="F254" t="s">
+        <v>610</v>
+      </c>
+      <c r="O254" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="255" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A255" t="s">
+        <v>875</v>
+      </c>
+      <c r="B255" t="s">
+        <v>884</v>
+      </c>
+      <c r="C255" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D255" t="s">
+        <v>926</v>
+      </c>
+      <c r="F255" t="s">
+        <v>610</v>
+      </c>
+      <c r="O255" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="256" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A256" t="s">
+        <v>876</v>
+      </c>
+      <c r="B256" t="s">
+        <v>884</v>
+      </c>
+      <c r="C256" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D256" t="s">
+        <v>927</v>
+      </c>
+      <c r="F256" t="s">
+        <v>610</v>
+      </c>
+      <c r="O256" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A257" t="s">
+        <v>877</v>
+      </c>
+      <c r="B257" t="s">
+        <v>884</v>
+      </c>
+      <c r="C257" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D257" t="s">
+        <v>928</v>
+      </c>
+      <c r="F257" t="s">
+        <v>610</v>
+      </c>
+      <c r="O257" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A258" t="s">
+        <v>878</v>
+      </c>
+      <c r="B258" t="s">
+        <v>884</v>
+      </c>
+      <c r="C258" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D258" t="s">
+        <v>929</v>
+      </c>
+      <c r="F258" t="s">
+        <v>610</v>
+      </c>
+      <c r="O258" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A259" t="s">
+        <v>879</v>
+      </c>
+      <c r="B259" t="s">
+        <v>894</v>
+      </c>
+      <c r="C259" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D259" t="s">
+        <v>930</v>
+      </c>
+      <c r="F259" t="s">
+        <v>610</v>
+      </c>
+      <c r="O259" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A260" t="s">
+        <v>880</v>
+      </c>
+      <c r="B260" t="s">
+        <v>884</v>
+      </c>
+      <c r="C260" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D260" t="s">
+        <v>931</v>
+      </c>
+      <c r="F260" t="s">
+        <v>610</v>
+      </c>
+      <c r="O260" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A261" t="s">
+        <v>881</v>
+      </c>
+      <c r="B261" t="s">
+        <v>884</v>
+      </c>
+      <c r="C261" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D261" t="s">
+        <v>932</v>
+      </c>
+      <c r="F261" t="s">
+        <v>610</v>
+      </c>
+      <c r="O261" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A262" t="s">
+        <v>882</v>
+      </c>
+      <c r="B262" t="s">
+        <v>884</v>
+      </c>
+      <c r="C262" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D262" t="s">
+        <v>933</v>
+      </c>
+      <c r="F262" t="s">
+        <v>610</v>
+      </c>
+      <c r="O262" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A263" t="s">
+        <v>883</v>
+      </c>
+      <c r="B263" t="s">
+        <v>884</v>
+      </c>
+      <c r="C263" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D263" t="s">
+        <v>934</v>
+      </c>
+      <c r="F263" t="s">
+        <v>610</v>
+      </c>
+      <c r="O263" s="14">
         <v>0</v>
       </c>
     </row>
@@ -11562,19 +12669,19 @@
     <cfRule type="duplicateValues" dxfId="39" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A107">
-    <cfRule type="duplicateValues" dxfId="38" priority="116"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="115"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="115"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="116"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A108:A110">
-    <cfRule type="duplicateValues" dxfId="36" priority="118"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="117"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="117"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="118"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A112:A134">
     <cfRule type="duplicateValues" dxfId="34" priority="119"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A138">
-    <cfRule type="duplicateValues" dxfId="33" priority="121"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="120"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="120"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="121"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A147:A155">
     <cfRule type="duplicateValues" dxfId="31" priority="122"/>
@@ -11624,8 +12731,8 @@
     <cfRule type="duplicateValues" dxfId="15" priority="86"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B140">
-    <cfRule type="duplicateValues" dxfId="14" priority="68"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B141">
     <cfRule type="duplicateValues" dxfId="12" priority="69"/>

</xml_diff>

<commit_message>
Weekly refresh — Tue 2026-07-07
SP-API pulls:
- FBA inbound Nexlev: 64 shipments / 108 rows (active-only)
- FBA inbound Viomi:  30 shipments / 102 rows (active-only)
- CB SOH: AA 142 ASINs / 11,273 units, Tonor 28 / 778
          SnapshotDate 2026-07-04

Operator updates: AA & WM Replenishment.xlsx + sku_master.xlsx.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
+++ b/data/input/Audio Array & WM Replenishment/AA & WM Replenishment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Audio Array &amp; WM Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2476F9D6-173C-4C5E-9AFB-64CF57A0789A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0EDE032-9C0E-4D71-8A62-37C06DB890BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E071ED51-FC72-421D-856E-2A4DF68E7BC3}"/>
   </bookViews>
@@ -2997,7 +2997,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12669,19 +12669,19 @@
     <cfRule type="duplicateValues" dxfId="39" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A107">
-    <cfRule type="duplicateValues" dxfId="38" priority="115"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A108:A110">
-    <cfRule type="duplicateValues" dxfId="36" priority="117"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="117"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A112:A134">
     <cfRule type="duplicateValues" dxfId="34" priority="119"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A138">
-    <cfRule type="duplicateValues" dxfId="33" priority="120"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="121"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="121"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="120"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A147:A155">
     <cfRule type="duplicateValues" dxfId="31" priority="122"/>
@@ -12731,8 +12731,8 @@
     <cfRule type="duplicateValues" dxfId="15" priority="86"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B140">
-    <cfRule type="duplicateValues" dxfId="14" priority="67"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B141">
     <cfRule type="duplicateValues" dxfId="12" priority="69"/>

</xml_diff>